<commit_message>
Persist firm portfolio with a stable id (approved trades now fill)
- FIRM_PORTFOLIO_ID stable constant; LedgerRepository.ensure_portfolio idempotent
- Live run + web runtime ensure + load the persisted portfolio (state persists
  across runs); _FakeLedger.ensure_portfolio no-op for offline
- Fixes 'Portfolio not found' on an approved buy; verified live (NVDA filled)
- +integration test; 395 tests green

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/2026-06-23.xlsx
+++ b/reports/2026-06-23.xlsx
@@ -462,19 +462,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>99999.69998799999</v>
+        <v>99999.754988</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.008731981719381119</v>
+        <v>-0.0121710358552735</v>
       </c>
       <c r="E2" t="n">
-        <v>0.008731981719381119</v>
+        <v>0.0121710358552735</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -521,17 +521,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="C2" t="n">
-        <v>373.2653717333333</v>
+        <v>201.700699</v>
       </c>
       <c r="D2" t="n">
-        <v>373.2653717333333</v>
+        <v>201.700699</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -548,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -597,6 +597,41 @@
           <t>ts</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>cd856b9a-9902-4f31-892a-cbbdb50e2de7</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>49</v>
+      </c>
+      <c r="E2" t="n">
+        <v>201.700699</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.93919753</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Human-in-the-loop on every cycle via Telegram, with override
- Always-HITL: risk node pauses every cycle (hitl_mode default 'always';
  threshold mode preserved). Human decides every cycle, not just big trades.
- resume_decision(approve/buy/sell/hold): approve executes the recommendation;
  reject lets the operator override; an override rewrites trade_proposal so
  synthesis/report/judge reflect what actually executed
- firm bot Telegram service: /run <ticker> -> rich card (recommendation, Why /
  Pros / Cons) -> Approve, or Reject -> Buy/Sell alternatives -> resume ->
  decision report + run report to the chat. Single getUpdates loop, non-blocking,
  durable via PostgresSaver (no webhook)
- research_manager leans buy-over-hold on borderline; Hold card shows 'no trade'
  (no phantom BUY 0); report labels distinguish approve vs override
- +117 tests (511 total); lint+mypy clean

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/2026-06-23.xlsx
+++ b/reports/2026-06-23.xlsx
@@ -462,19 +462,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>99999.754988</v>
+        <v>99920.92971647851</v>
       </c>
       <c r="C2" t="n">
+        <v>-78.75527752148406</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-0.01386371004599338</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.01307553405779002</v>
+      </c>
+      <c r="F2" t="n">
         <v>0</v>
-      </c>
-      <c r="D2" t="n">
-        <v>-0.0121710358552735</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.0121710358552735</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -525,16 +525,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="C2" t="n">
-        <v>201.700699</v>
+        <v>201.5250776666667</v>
       </c>
       <c r="D2" t="n">
-        <v>201.700699</v>
+        <v>200.2749938964844</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>-78.75527752148406</v>
       </c>
     </row>
   </sheetData>
@@ -548,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -597,41 +597,6 @@
           <t>ts</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>cd856b9a-9902-4f31-892a-cbbdb50e2de7</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>NVDA</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>buy</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>49</v>
-      </c>
-      <c r="E2" t="n">
-        <v>201.700699</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4.93919753</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.245</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>FILLED</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>